<commit_message>
Added sound attribution to credits
</commit_message>
<xml_diff>
--- a/Other/Sounds.xlsx
+++ b/Other/Sounds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/623821e34d642ca0/Desktop/ASVGC-25/Other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{8189D8F4-1E64-4DF1-B2A6-68F1B77D596A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8013C73C-A333-403F-8172-AAA97A9F18EF}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="8_{8189D8F4-1E64-4DF1-B2A6-68F1B77D596A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F11BE50-D9C3-4ACE-9637-F5DE17D898A9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{53BCC81A-2A92-4691-9841-E4BA723E9FDD}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{53BCC81A-2A92-4691-9841-E4BA723E9FDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>